<commit_message>
[V4 A] xong report_full
</commit_message>
<xml_diff>
--- a/results/gnn_rl/bang_tong_hop_gnn_rl.xlsx
+++ b/results/gnn_rl/bang_tong_hop_gnn_rl.xlsx
@@ -1354,7 +1354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1747,54 +1747,54 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>branch_odgraphformer</t>
+          <t>rl_sac_no_oof</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>0.7856831775612649</v>
+        <v>0.7218451636614334</v>
       </c>
       <c r="E7" t="n">
-        <v>5.887070317139143</v>
+        <v>5.455012669519333</v>
       </c>
       <c r="F7" t="n">
-        <v>0.5178367351444001</v>
+        <v>0.4471953363100333</v>
       </c>
       <c r="G7" t="n">
-        <v>0.3107024173756095</v>
+        <v>0.3132705326157333</v>
       </c>
       <c r="H7" t="n">
-        <v>0.8694401492276453</v>
+        <v>0.8612424204224908</v>
       </c>
       <c r="I7" t="n">
-        <v>0.6240313550206674</v>
+        <v>0.8094240791732087</v>
       </c>
       <c r="J7" t="n">
-        <v>0.01041224897936075</v>
+        <v>0.005877267269421888</v>
       </c>
       <c r="K7" t="n">
-        <v>0.2274492561295375</v>
+        <v>0.03145793899763993</v>
       </c>
       <c r="L7" t="n">
-        <v>0.007818188448588366</v>
+        <v>0.000585589696054073</v>
       </c>
       <c r="M7" t="n">
-        <v>0.0003525583492634219</v>
+        <v>0.000801606758211442</v>
       </c>
       <c r="N7" t="n">
-        <v>0.002671004988153148</v>
+        <v>0.001420777978255195</v>
       </c>
       <c r="O7" t="n">
-        <v>0.01458200086210178</v>
+        <v>0.001784030015620982</v>
       </c>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>OD-GraphFormer đầy đủ</t>
+          <t>RL-Gate: không dùng OOF</t>
         </is>
       </c>
     </row>
@@ -1806,52 +1806,111 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>branch_odgraphformer</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.7856831775612649</v>
+      </c>
+      <c r="E8" t="n">
+        <v>5.887070317139143</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.5178367351444001</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.3107024173756095</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.8694401492276453</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.6240313550206674</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.01041224897936075</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.2274492561295375</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.007818188448588366</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.0003525583492634219</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.002671004988153148</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.01458200086210178</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>OD-GraphFormer đầy đủ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>geant</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>rl_sac</t>
         </is>
       </c>
-      <c r="C8" t="n">
-        <v>3</v>
-      </c>
-      <c r="D8" t="n">
+      <c r="C9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" t="n">
         <v>0.7225773738886001</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E9" t="n">
         <v>5.452208487349799</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F9" t="n">
         <v>0.4472464966468</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G9" t="n">
         <v>0.3135579154232334</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H9" t="n">
         <v>0.8613959983095422</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I9" t="n">
         <v>0.8094781804549888</v>
       </c>
-      <c r="J8" t="n">
+      <c r="J9" t="n">
         <v>0.006392578699177021</v>
       </c>
-      <c r="K8" t="n">
+      <c r="K9" t="n">
         <v>0.03434962783607208</v>
       </c>
-      <c r="L8" t="n">
+      <c r="L9" t="n">
         <v>0.0007994427614239256</v>
       </c>
-      <c r="M8" t="n">
+      <c r="M9" t="n">
         <v>0.0008496145493271741</v>
       </c>
-      <c r="N8" t="n">
+      <c r="N9" t="n">
         <v>0.001506649409099997</v>
       </c>
-      <c r="O8" t="n">
+      <c r="O9" t="n">
         <v>0.002192561491826783</v>
       </c>
-      <c r="P8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" t="inlineStr">
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="inlineStr">
         <is>
           <t>RL-Gate đầy đủ</t>
         </is>

</xml_diff>

<commit_message>
[V4 B] xong report_full
</commit_message>
<xml_diff>
--- a/results/gnn_rl/bang_tong_hop_gnn_rl.xlsx
+++ b/results/gnn_rl/bang_tong_hop_gnn_rl.xlsx
@@ -2180,7 +2180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2455,54 +2455,54 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>branch_odgraphformer</t>
+          <t>rl_sac_no_gnn</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>3</v>
       </c>
       <c r="D5" t="n">
-        <v>1.928859386545132</v>
+        <v>1.8483099679539</v>
       </c>
       <c r="E5" t="n">
-        <v>16.81178907153938</v>
+        <v>16.2707895666414</v>
       </c>
       <c r="F5" t="n">
-        <v>1.362165365616967</v>
+        <v>1.312961791312367</v>
       </c>
       <c r="G5" t="n">
-        <v>1.152399188611637</v>
+        <v>1.0295819927706</v>
       </c>
       <c r="H5" t="n">
-        <v>0.6685984633630261</v>
+        <v>0.6862377355285362</v>
       </c>
       <c r="I5" t="n">
-        <v>0.650800530080651</v>
+        <v>0.6565687596501162</v>
       </c>
       <c r="J5" t="n">
-        <v>0.01545501552364565</v>
+        <v>0.02231784771708809</v>
       </c>
       <c r="K5" t="n">
-        <v>0.004620099755121902</v>
+        <v>0.02017964382671037</v>
       </c>
       <c r="L5" t="n">
-        <v>0.01624505993671197</v>
+        <v>0.04532015910518247</v>
       </c>
       <c r="M5" t="n">
-        <v>0.01678374989219983</v>
+        <v>0.01872892072531651</v>
       </c>
       <c r="N5" t="n">
-        <v>0.002736130749175138</v>
+        <v>0.00340463964995482</v>
       </c>
       <c r="O5" t="n">
-        <v>0.008094133189538432</v>
+        <v>0.02741506628518012</v>
       </c>
       <c r="P5" t="n">
         <v>0</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>OD-GraphFormer đầy đủ</t>
+          <t>RL-Gate: bỏ GNN</t>
         </is>
       </c>
     </row>
@@ -2514,231 +2514,231 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>rl_sac</t>
+          <t>rl_sac_no_floor</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>3</v>
       </c>
       <c r="D6" t="n">
-        <v>1.855865671600433</v>
+        <v>1.853823748186333</v>
       </c>
       <c r="E6" t="n">
-        <v>16.2774170290789</v>
+        <v>16.27837458257217</v>
       </c>
       <c r="F6" t="n">
-        <v>1.3335921242009</v>
+        <v>1.330673950370433</v>
       </c>
       <c r="G6" t="n">
-        <v>1.018908983414767</v>
+        <v>1.019692554900267</v>
       </c>
       <c r="H6" t="n">
-        <v>0.6873266992176704</v>
+        <v>0.6868896527036062</v>
       </c>
       <c r="I6" t="n">
-        <v>0.6440014459931426</v>
+        <v>0.6460493397521928</v>
       </c>
       <c r="J6" t="n">
-        <v>0.007077109341909518</v>
+        <v>0.007448525828711058</v>
       </c>
       <c r="K6" t="n">
-        <v>0.01378671369864897</v>
+        <v>0.01248625361193996</v>
       </c>
       <c r="L6" t="n">
-        <v>0.006439372149233406</v>
+        <v>0.006911682539066343</v>
       </c>
       <c r="M6" t="n">
-        <v>0.005697519008396951</v>
+        <v>0.005076647640855694</v>
       </c>
       <c r="N6" t="n">
-        <v>0.001003724468154216</v>
+        <v>0.0009236603046667447</v>
       </c>
       <c r="O6" t="n">
-        <v>0.003020044501720799</v>
+        <v>0.002936888568788178</v>
       </c>
       <c r="P6" t="n">
         <v>0</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>RL-Gate đầy đủ</t>
+          <t>RL-Gate: bỏ ràng buộc sàn</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>abilene</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>odgraphformer_no_residual</t>
+          <t>rl_sac_no_oof</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>4.8276139688106</v>
+        <v>1.855546859557733</v>
       </c>
       <c r="E7" t="n">
-        <v>41.5047214284323</v>
+        <v>16.2766456073441</v>
       </c>
       <c r="F7" t="n">
-        <v>4.748738791231708</v>
+        <v>1.3331067956906</v>
       </c>
       <c r="G7" t="n">
-        <v>4.748759486366427</v>
+        <v>1.0188396173319</v>
       </c>
       <c r="H7" t="n">
-        <v>0.2963983477427541</v>
+        <v>0.687307561792645</v>
       </c>
       <c r="I7" t="n">
-        <v>0.5299587290167037</v>
+        <v>0.6442105130749479</v>
       </c>
       <c r="J7" t="n">
-        <v>0.2357659810412736</v>
+        <v>0.006795330218235516</v>
       </c>
       <c r="K7" t="n">
-        <v>1.023521497138683</v>
+        <v>0.01269511918196406</v>
       </c>
       <c r="L7" t="n">
-        <v>0.2375486340469883</v>
+        <v>0.006071805603038467</v>
       </c>
       <c r="M7" t="n">
-        <v>0.2362353370503212</v>
+        <v>0.005341100850855931</v>
       </c>
       <c r="N7" t="n">
-        <v>0.006027497320855425</v>
+        <v>0.0009691001253040893</v>
       </c>
       <c r="O7" t="n">
-        <v>0.01153529849583505</v>
+        <v>0.002864999433636739</v>
       </c>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>OD-GraphFormer: bỏ mục tiêu phần dư</t>
+          <t>RL-Gate: không dùng OOF</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>abilene</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>odgraphformer_no_route</t>
+          <t>branch_odgraphformer</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>10.66293271400805</v>
+        <v>1.928859386545132</v>
       </c>
       <c r="E8" t="n">
-        <v>60.30897322814824</v>
+        <v>16.81178907153938</v>
       </c>
       <c r="F8" t="n">
-        <v>10.5588699804009</v>
+        <v>1.362165365616967</v>
       </c>
       <c r="G8" t="n">
-        <v>10.40103781037437</v>
+        <v>1.152399188611637</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2632649427674279</v>
+        <v>0.6685984633630261</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6470081480990179</v>
+        <v>0.650800530080651</v>
       </c>
       <c r="J8" t="n">
-        <v>0.08053701985678052</v>
+        <v>0.01545501552364565</v>
       </c>
       <c r="K8" t="n">
-        <v>0.2267106013798933</v>
+        <v>0.004620099755121902</v>
       </c>
       <c r="L8" t="n">
-        <v>0.08002285928659564</v>
+        <v>0.01624505993671197</v>
       </c>
       <c r="M8" t="n">
-        <v>0.06990591943031775</v>
+        <v>0.01678374989219983</v>
       </c>
       <c r="N8" t="n">
-        <v>0.002663265318122867</v>
+        <v>0.002736130749175138</v>
       </c>
       <c r="O8" t="n">
-        <v>0.001422903613711275</v>
+        <v>0.008094133189538432</v>
       </c>
       <c r="P8" t="n">
         <v>0</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>OD-GraphFormer: bỏ A_route</t>
+          <t>OD-GraphFormer đầy đủ</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>abilene</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>odgraphformer_no_spatial_attn</t>
+          <t>rl_sac</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>10.9102780209387</v>
+        <v>1.855865671600433</v>
       </c>
       <c r="E9" t="n">
-        <v>61.18399339636263</v>
+        <v>16.2774170290789</v>
       </c>
       <c r="F9" t="n">
-        <v>10.80425328520641</v>
+        <v>1.3335921242009</v>
       </c>
       <c r="G9" t="n">
-        <v>10.63499236387419</v>
+        <v>1.018908983414767</v>
       </c>
       <c r="H9" t="n">
-        <v>0.2635857497749368</v>
+        <v>0.6873266992176704</v>
       </c>
       <c r="I9" t="n">
-        <v>0.6659195441296032</v>
+        <v>0.6440014459931426</v>
       </c>
       <c r="J9" t="n">
-        <v>0.066160960598211</v>
+        <v>0.007077109341909518</v>
       </c>
       <c r="K9" t="n">
-        <v>0.1883156720439629</v>
+        <v>0.01378671369864897</v>
       </c>
       <c r="L9" t="n">
-        <v>0.06655299041987504</v>
+        <v>0.006439372149233406</v>
       </c>
       <c r="M9" t="n">
-        <v>0.04785879943660532</v>
+        <v>0.005697519008396951</v>
       </c>
       <c r="N9" t="n">
-        <v>0.00395845662169573</v>
+        <v>0.001003724468154216</v>
       </c>
       <c r="O9" t="n">
-        <v>0.01444244036559092</v>
+        <v>0.003020044501720799</v>
       </c>
       <c r="P9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>OD-GraphFormer: bỏ attention giữa luồng</t>
+          <t>RL-Gate đầy đủ</t>
         </is>
       </c>
     </row>
@@ -2750,54 +2750,54 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>rl_sac_no_floor</t>
+          <t>odgraphformer_no_residual</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>4.528418422798134</v>
+        <v>4.8276139688106</v>
       </c>
       <c r="E10" t="n">
-        <v>39.09603904405284</v>
+        <v>41.5047214284323</v>
       </c>
       <c r="F10" t="n">
-        <v>4.4259005183743</v>
+        <v>4.748738791231708</v>
       </c>
       <c r="G10" t="n">
-        <v>4.389191853846733</v>
+        <v>4.748759486366427</v>
       </c>
       <c r="H10" t="n">
-        <v>0.3421658448997631</v>
+        <v>0.2963983477427541</v>
       </c>
       <c r="I10" t="n">
-        <v>0.5692215955020613</v>
+        <v>0.5299587290167037</v>
       </c>
       <c r="J10" t="n">
-        <v>0.0162723717959731</v>
+        <v>0.2357659810412736</v>
       </c>
       <c r="K10" t="n">
-        <v>0.1207024858161245</v>
+        <v>1.023521497138683</v>
       </c>
       <c r="L10" t="n">
-        <v>0.01652362515098457</v>
+        <v>0.2375486340469883</v>
       </c>
       <c r="M10" t="n">
-        <v>0.01763783668073158</v>
+        <v>0.2362353370503212</v>
       </c>
       <c r="N10" t="n">
-        <v>0.001514510517106802</v>
+        <v>0.006027497320855425</v>
       </c>
       <c r="O10" t="n">
-        <v>0.00548192115092797</v>
+        <v>0.01153529849583505</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>RL-Gate: bỏ ràng buộc sàn</t>
+          <t>OD-GraphFormer: bỏ mục tiêu phần dư</t>
         </is>
       </c>
     </row>
@@ -2809,54 +2809,54 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>branch_odgraphformer</t>
+          <t>odgraphformer_no_route</t>
         </is>
       </c>
       <c r="C11" t="n">
         <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>10.82378673206354</v>
+        <v>10.66293271400805</v>
       </c>
       <c r="E11" t="n">
-        <v>60.98440293556504</v>
+        <v>60.30897322814824</v>
       </c>
       <c r="F11" t="n">
-        <v>10.71875904785843</v>
+        <v>10.5588699804009</v>
       </c>
       <c r="G11" t="n">
-        <v>10.55165324861514</v>
+        <v>10.40103781037437</v>
       </c>
       <c r="H11" t="n">
-        <v>0.2656305682531275</v>
+        <v>0.2632649427674279</v>
       </c>
       <c r="I11" t="n">
-        <v>0.653468604478941</v>
+        <v>0.6470081480990179</v>
       </c>
       <c r="J11" t="n">
-        <v>0.5172167404793825</v>
+        <v>0.08053701985678052</v>
       </c>
       <c r="K11" t="n">
-        <v>1.426460798016727</v>
+        <v>0.2267106013798933</v>
       </c>
       <c r="L11" t="n">
-        <v>0.5149674442874014</v>
+        <v>0.08002285928659564</v>
       </c>
       <c r="M11" t="n">
-        <v>0.4916759040166223</v>
+        <v>0.06990591943031775</v>
       </c>
       <c r="N11" t="n">
-        <v>0.00122086714363905</v>
+        <v>0.002663265318122867</v>
       </c>
       <c r="O11" t="n">
-        <v>0.01292813018908067</v>
+        <v>0.001422903613711275</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>OD-GraphFormer đầy đủ</t>
+          <t>OD-GraphFormer: bỏ A_route</t>
         </is>
       </c>
     </row>
@@ -2868,52 +2868,347 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>odgraphformer_no_spatial_attn</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" t="n">
+        <v>10.9102780209387</v>
+      </c>
+      <c r="E12" t="n">
+        <v>61.18399339636263</v>
+      </c>
+      <c r="F12" t="n">
+        <v>10.80425328520641</v>
+      </c>
+      <c r="G12" t="n">
+        <v>10.63499236387419</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.2635857497749368</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.6659195441296032</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.066160960598211</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.1883156720439629</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.06655299041987504</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.04785879943660532</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.00395845662169573</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.01444244036559092</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>OD-GraphFormer: bỏ attention giữa luồng</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>rl_sac_no_gnn</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" t="n">
+        <v>4.6007980620559</v>
+      </c>
+      <c r="E13" t="n">
+        <v>39.4685735956757</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4.497778798865401</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4.483965509299467</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.3366507029696833</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.582159349679667</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.03924523452740855</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.2237184556650453</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.03949077697060992</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.03871445401052525</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.001850556307376831</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.003245605516320773</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>RL-Gate: bỏ GNN</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>rl_sac_no_floor</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" t="n">
+        <v>4.528418422798134</v>
+      </c>
+      <c r="E14" t="n">
+        <v>39.09603904405284</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4.4259005183743</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4.389191853846733</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.3421658448997631</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.5692215955020613</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.0162723717959731</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.1207024858161245</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.01652362515098457</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.01763783668073158</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0.001514510517106802</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.00548192115092797</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>RL-Gate: bỏ ràng buộc sàn</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>rl_sac_no_oof</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" t="n">
+        <v>4.710557639548266</v>
+      </c>
+      <c r="E15" t="n">
+        <v>40.06596057594567</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4.608354158853033</v>
+      </c>
+      <c r="G15" t="n">
+        <v>4.589994634922399</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.3321333617750766</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.5812170010577616</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.1769022240669252</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.787068196298402</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.1763398443973145</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.177536843462079</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.004822580596551231</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.008334709652361447</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>RL-Gate: không dùng OOF</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>branch_odgraphformer</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" t="n">
+        <v>10.82378673206354</v>
+      </c>
+      <c r="E16" t="n">
+        <v>60.98440293556504</v>
+      </c>
+      <c r="F16" t="n">
+        <v>10.71875904785843</v>
+      </c>
+      <c r="G16" t="n">
+        <v>10.55165324861514</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.2656305682531275</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.653468604478941</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.5172167404793825</v>
+      </c>
+      <c r="K16" t="n">
+        <v>1.426460798016727</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.5149674442874014</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.4916759040166223</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0.00122086714363905</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.01292813018908067</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>OD-GraphFormer đầy đủ</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>rl_sac</t>
         </is>
       </c>
-      <c r="C12" t="n">
-        <v>3</v>
-      </c>
-      <c r="D12" t="n">
+      <c r="C17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" t="n">
         <v>4.480196253950034</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E17" t="n">
         <v>38.89223448794053</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F17" t="n">
         <v>4.378142004008133</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G17" t="n">
         <v>4.344089959168966</v>
       </c>
-      <c r="H12" t="n">
+      <c r="H17" t="n">
         <v>0.3427342928399741</v>
       </c>
-      <c r="I12" t="n">
+      <c r="I17" t="n">
         <v>0.5839717434300823</v>
       </c>
-      <c r="J12" t="n">
+      <c r="J17" t="n">
         <v>0.03348693805469789</v>
       </c>
-      <c r="K12" t="n">
+      <c r="K17" t="n">
         <v>0.2008306145023352</v>
       </c>
-      <c r="L12" t="n">
+      <c r="L17" t="n">
         <v>0.03296962066273203</v>
       </c>
-      <c r="M12" t="n">
+      <c r="M17" t="n">
         <v>0.03573225124601732</v>
       </c>
-      <c r="N12" t="n">
+      <c r="N17" t="n">
         <v>0.002119665720671422</v>
       </c>
-      <c r="O12" t="n">
+      <c r="O17" t="n">
         <v>0.007700102234067678</v>
       </c>
-      <c r="P12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" t="inlineStr">
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="inlineStr">
         <is>
           <t>RL-Gate đầy đủ</t>
         </is>

</xml_diff>

<commit_message>
[V4 B] gộp A + B, báo cáo chung
</commit_message>
<xml_diff>
--- a/results/gnn_rl/bang_tong_hop_gnn_rl.xlsx
+++ b/results/gnn_rl/bang_tong_hop_gnn_rl.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q29"/>
+  <dimension ref="A1:Q43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1346,7 +1346,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1358,22 +1358,22 @@
         <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>26.55449157545777</v>
+        <v>0.8545949154731397</v>
       </c>
       <c r="E16" t="n">
-        <v>90.96799341654842</v>
+        <v>5.632607437995413</v>
       </c>
       <c r="F16" t="n">
-        <v>26.42186862643311</v>
+        <v>0.5819590981680846</v>
       </c>
       <c r="G16" t="n">
-        <v>25.69528161983637</v>
+        <v>0.339302939314644</v>
       </c>
       <c r="H16" t="n">
-        <v>0.2110912108471329</v>
+        <v>0.8691391710779487</v>
       </c>
       <c r="I16" t="n">
-        <v>0.4498484483944032</v>
+        <v>0.5329569135522744</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1417,40 +1417,40 @@
         <v>3</v>
       </c>
       <c r="D17" t="n">
-        <v>5.501746132110231</v>
+        <v>0.9160362802011897</v>
       </c>
       <c r="E17" t="n">
-        <v>43.50135691079012</v>
+        <v>5.864958530080304</v>
       </c>
       <c r="F17" t="n">
-        <v>5.400941108775661</v>
+        <v>0.4552296270502245</v>
       </c>
       <c r="G17" t="n">
-        <v>5.38897000852714</v>
+        <v>0.3443731357643805</v>
       </c>
       <c r="H17" t="n">
-        <v>0.3104524120407648</v>
+        <v>0.8797340421617648</v>
       </c>
       <c r="I17" t="n">
-        <v>0.5979225042188075</v>
+        <v>0.7289891544548174</v>
       </c>
       <c r="J17" t="n">
-        <v>0.03648634416566095</v>
+        <v>0.001991306910794514</v>
       </c>
       <c r="K17" t="n">
-        <v>0.1800025294142001</v>
+        <v>0.003753233538075241</v>
       </c>
       <c r="L17" t="n">
-        <v>0.03583735584964644</v>
+        <v>0.000699093897774393</v>
       </c>
       <c r="M17" t="n">
-        <v>0.03555507731483454</v>
+        <v>0.0006337084715600187</v>
       </c>
       <c r="N17" t="n">
-        <v>0.002514829252129105</v>
+        <v>0.0004551147754948264</v>
       </c>
       <c r="O17" t="n">
-        <v>0.008006618946304844</v>
+        <v>0.0004809586111362458</v>
       </c>
       <c r="P17" t="n">
         <v>0</v>
@@ -1464,7 +1464,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1476,40 +1476,40 @@
         <v>3</v>
       </c>
       <c r="D18" t="n">
-        <v>4.725293687942619</v>
+        <v>0.7511689919265434</v>
       </c>
       <c r="E18" t="n">
-        <v>40.09050711039001</v>
+        <v>5.755513447990891</v>
       </c>
       <c r="F18" t="n">
-        <v>4.622366665383944</v>
+        <v>0.4643777229002375</v>
       </c>
       <c r="G18" t="n">
-        <v>4.58088827254178</v>
+        <v>0.3101534872891977</v>
       </c>
       <c r="H18" t="n">
-        <v>0.3346154045021904</v>
+        <v>0.863424599693689</v>
       </c>
       <c r="I18" t="n">
-        <v>0.5685760891694658</v>
+        <v>0.7024949865466629</v>
       </c>
       <c r="J18" t="n">
-        <v>0.04001095344222513</v>
+        <v>0.0007415452738515091</v>
       </c>
       <c r="K18" t="n">
-        <v>0.2356779729660841</v>
+        <v>0.006526737487821046</v>
       </c>
       <c r="L18" t="n">
-        <v>0.04040968708202303</v>
+        <v>0.0009672950477639932</v>
       </c>
       <c r="M18" t="n">
-        <v>0.04102459753013328</v>
+        <v>0.0005450964630930178</v>
       </c>
       <c r="N18" t="n">
-        <v>0.002412511766822248</v>
+        <v>0.000335233721423481</v>
       </c>
       <c r="O18" t="n">
-        <v>0.003194804001046742</v>
+        <v>0.00137040939017097</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1523,7 +1523,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1535,40 +1535,40 @@
         <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>15.05727505024088</v>
+        <v>0.7362113194966695</v>
       </c>
       <c r="E19" t="n">
-        <v>64.31187253033912</v>
+        <v>5.399883671026634</v>
       </c>
       <c r="F19" t="n">
-        <v>14.95331586609725</v>
+        <v>0.4686869846584136</v>
       </c>
       <c r="G19" t="n">
-        <v>14.62828864718621</v>
+        <v>0.325092830932584</v>
       </c>
       <c r="H19" t="n">
-        <v>0.3033576975106618</v>
+        <v>0.8610793040993343</v>
       </c>
       <c r="I19" t="n">
-        <v>0.7939136373143997</v>
+        <v>0.7934766876314812</v>
       </c>
       <c r="J19" t="n">
-        <v>0.3879300898569781</v>
+        <v>0.007013931251638423</v>
       </c>
       <c r="K19" t="n">
-        <v>1.442674289781311</v>
+        <v>0.009629990920579486</v>
       </c>
       <c r="L19" t="n">
-        <v>0.3902316522193149</v>
+        <v>0.001906264768356159</v>
       </c>
       <c r="M19" t="n">
-        <v>0.3791228986791557</v>
+        <v>0.002963214704868111</v>
       </c>
       <c r="N19" t="n">
-        <v>0.007868257797702578</v>
+        <v>0.002152269993402452</v>
       </c>
       <c r="O19" t="n">
-        <v>0.006935287930042821</v>
+        <v>0.004500665234824578</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
@@ -1582,7 +1582,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1594,40 +1594,40 @@
         <v>3</v>
       </c>
       <c r="D20" t="n">
-        <v>10.82378673206354</v>
+        <v>0.7856831775612649</v>
       </c>
       <c r="E20" t="n">
-        <v>60.98440293556504</v>
+        <v>5.887070317139143</v>
       </c>
       <c r="F20" t="n">
-        <v>10.71875904785843</v>
+        <v>0.5178367351444001</v>
       </c>
       <c r="G20" t="n">
-        <v>10.55165324861514</v>
+        <v>0.3107024173756095</v>
       </c>
       <c r="H20" t="n">
-        <v>0.2656305682531275</v>
+        <v>0.8694401492276453</v>
       </c>
       <c r="I20" t="n">
-        <v>0.653468604478941</v>
+        <v>0.6240313550206674</v>
       </c>
       <c r="J20" t="n">
-        <v>0.5172167404793825</v>
+        <v>0.01041224897936075</v>
       </c>
       <c r="K20" t="n">
-        <v>1.426460798016727</v>
+        <v>0.2274492561295375</v>
       </c>
       <c r="L20" t="n">
-        <v>0.5149674442874014</v>
+        <v>0.007818188448588366</v>
       </c>
       <c r="M20" t="n">
-        <v>0.4916759040166223</v>
+        <v>0.0003525583492634219</v>
       </c>
       <c r="N20" t="n">
-        <v>0.00122086714363905</v>
+        <v>0.002671004988153148</v>
       </c>
       <c r="O20" t="n">
-        <v>0.01292813018908067</v>
+        <v>0.01458200086210178</v>
       </c>
       <c r="P20" t="n">
         <v>0</v>
@@ -1641,7 +1641,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1653,40 +1653,40 @@
         <v>3</v>
       </c>
       <c r="D21" t="n">
-        <v>4.016685571412967</v>
+        <v>0.7235077901182334</v>
       </c>
       <c r="E21" t="n">
-        <v>38.12959362032276</v>
+        <v>5.456814616815633</v>
       </c>
       <c r="F21" t="n">
-        <v>3.9141140577925</v>
+        <v>0.4468465863660333</v>
       </c>
       <c r="G21" t="n">
-        <v>3.881554694383667</v>
+        <v>0.3137544199187</v>
       </c>
       <c r="H21" t="n">
-        <v>0.3216286447809846</v>
+        <v>0.8614537406438583</v>
       </c>
       <c r="I21" t="n">
-        <v>0.6358823934634544</v>
+        <v>0.8109079800947187</v>
       </c>
       <c r="J21" t="n">
-        <v>0.0511924947251717</v>
+        <v>0.005211460970558278</v>
       </c>
       <c r="K21" t="n">
-        <v>0.2919558767863844</v>
+        <v>0.03228928404691184</v>
       </c>
       <c r="L21" t="n">
-        <v>0.05138622364983586</v>
+        <v>0.0001647485566469421</v>
       </c>
       <c r="M21" t="n">
-        <v>0.05120899677502607</v>
+        <v>0.0007953819053387523</v>
       </c>
       <c r="N21" t="n">
-        <v>0.002258133129645119</v>
+        <v>0.001500156802479793</v>
       </c>
       <c r="O21" t="n">
-        <v>0.002740557556229231</v>
+        <v>0.0003630989720368629</v>
       </c>
       <c r="P21" t="n">
         <v>0</v>
@@ -1700,7 +1700,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1712,40 +1712,40 @@
         <v>3</v>
       </c>
       <c r="D22" t="n">
-        <v>4.0006725430085</v>
+        <v>0.7234406460867</v>
       </c>
       <c r="E22" t="n">
-        <v>38.04336307929087</v>
+        <v>5.4569258729912</v>
       </c>
       <c r="F22" t="n">
-        <v>3.898104438271266</v>
+        <v>0.4468731408295333</v>
       </c>
       <c r="G22" t="n">
-        <v>3.865385824036534</v>
+        <v>0.3137071902637333</v>
       </c>
       <c r="H22" t="n">
-        <v>0.3221728402357322</v>
+        <v>0.8614435703170424</v>
       </c>
       <c r="I22" t="n">
-        <v>0.6361394316594257</v>
+        <v>0.8107993502951963</v>
       </c>
       <c r="J22" t="n">
-        <v>0.05083442098161815</v>
+        <v>0.005211220671549527</v>
       </c>
       <c r="K22" t="n">
-        <v>0.2936563955059048</v>
+        <v>0.03232065102623457</v>
       </c>
       <c r="L22" t="n">
-        <v>0.05101751928635763</v>
+        <v>0.0001650355779724377</v>
       </c>
       <c r="M22" t="n">
-        <v>0.05081318515054815</v>
+        <v>0.0007956009324682908</v>
       </c>
       <c r="N22" t="n">
-        <v>0.002170762595070282</v>
+        <v>0.001498680412343242</v>
       </c>
       <c r="O22" t="n">
-        <v>0.002791217678190753</v>
+        <v>0.0003605477777677723</v>
       </c>
       <c r="P22" t="n">
         <v>3</v>
@@ -1759,7 +1759,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1771,40 +1771,40 @@
         <v>3</v>
       </c>
       <c r="D23" t="n">
-        <v>4.684722348874001</v>
+        <v>0.7235080178355666</v>
       </c>
       <c r="E23" t="n">
-        <v>39.83803320540737</v>
+        <v>5.456815081481034</v>
       </c>
       <c r="F23" t="n">
-        <v>4.582328381558233</v>
+        <v>0.44684653536</v>
       </c>
       <c r="G23" t="n">
-        <v>4.553032977087266</v>
+        <v>0.3137544712419667</v>
       </c>
       <c r="H23" t="n">
-        <v>0.3361538283555277</v>
+        <v>0.8614537623223063</v>
       </c>
       <c r="I23" t="n">
-        <v>0.5760268776804347</v>
+        <v>0.8109081106406428</v>
       </c>
       <c r="J23" t="n">
-        <v>0.04131775529316326</v>
+        <v>0.005211556523500392</v>
       </c>
       <c r="K23" t="n">
-        <v>0.2329841362440988</v>
+        <v>0.03228888884369236</v>
       </c>
       <c r="L23" t="n">
-        <v>0.04150812133718134</v>
+        <v>0.0001647298033946594</v>
       </c>
       <c r="M23" t="n">
-        <v>0.04148202553812069</v>
+        <v>0.0007954248742274059</v>
       </c>
       <c r="N23" t="n">
-        <v>0.002092411740696855</v>
+        <v>0.001500174092446543</v>
       </c>
       <c r="O23" t="n">
-        <v>0.004240845807268545</v>
+        <v>0.0003630051104621055</v>
       </c>
       <c r="P23" t="n">
         <v>0</v>
@@ -1818,7 +1818,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1830,40 +1830,40 @@
         <v>3</v>
       </c>
       <c r="D24" t="n">
-        <v>4.542170142965533</v>
+        <v>0.7509228569232</v>
       </c>
       <c r="E24" t="n">
-        <v>39.2482763158854</v>
+        <v>5.476798487561567</v>
       </c>
       <c r="F24" t="n">
-        <v>4.439539794282</v>
+        <v>0.4530580908306333</v>
       </c>
       <c r="G24" t="n">
-        <v>4.422377569527034</v>
+        <v>0.3096083548637666</v>
       </c>
       <c r="H24" t="n">
-        <v>0.3365139811403686</v>
+        <v>0.8667797937050526</v>
       </c>
       <c r="I24" t="n">
-        <v>0.5854458781691547</v>
+        <v>0.7498925451143607</v>
       </c>
       <c r="J24" t="n">
-        <v>0.03842453494253652</v>
+        <v>0.006005240601259012</v>
       </c>
       <c r="K24" t="n">
-        <v>0.2001784443270455</v>
+        <v>0.02169411228162643</v>
       </c>
       <c r="L24" t="n">
-        <v>0.03870985882774151</v>
+        <v>0.002751827371387717</v>
       </c>
       <c r="M24" t="n">
-        <v>0.03720438800025542</v>
+        <v>0.0001239548096339272</v>
       </c>
       <c r="N24" t="n">
-        <v>0.001478039886136305</v>
+        <v>0.001177476155245675</v>
       </c>
       <c r="O24" t="n">
-        <v>0.003967245799738929</v>
+        <v>0.005477748418061815</v>
       </c>
       <c r="P24" t="n">
         <v>0</v>
@@ -1877,7 +1877,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1889,40 +1889,40 @@
         <v>3</v>
       </c>
       <c r="D25" t="n">
-        <v>4.542170142965533</v>
+        <v>0.7319333071974</v>
       </c>
       <c r="E25" t="n">
-        <v>39.2482763158854</v>
+        <v>5.460561931117267</v>
       </c>
       <c r="F25" t="n">
-        <v>4.439539794282</v>
+        <v>0.4492073240654</v>
       </c>
       <c r="G25" t="n">
-        <v>4.422377569527034</v>
+        <v>0.3092457194735</v>
       </c>
       <c r="H25" t="n">
-        <v>0.3365139811403686</v>
+        <v>0.8636356837478868</v>
       </c>
       <c r="I25" t="n">
-        <v>0.5854458781691547</v>
+        <v>0.7792759342320341</v>
       </c>
       <c r="J25" t="n">
-        <v>0.03842453494253652</v>
+        <v>0.008363037458121574</v>
       </c>
       <c r="K25" t="n">
-        <v>0.2001784443270455</v>
+        <v>0.02779811631458437</v>
       </c>
       <c r="L25" t="n">
-        <v>0.03870985882774151</v>
+        <v>0.003128744893328703</v>
       </c>
       <c r="M25" t="n">
-        <v>0.03720438800025542</v>
+        <v>0.0001529779934639351</v>
       </c>
       <c r="N25" t="n">
-        <v>0.001478039886136305</v>
+        <v>0.001281465881999977</v>
       </c>
       <c r="O25" t="n">
-        <v>0.003967245799738929</v>
+        <v>0.0123427233725683</v>
       </c>
       <c r="P25" t="n">
         <v>0</v>
@@ -1936,7 +1936,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1948,40 +1948,40 @@
         <v>3</v>
       </c>
       <c r="D26" t="n">
-        <v>4.686588991352133</v>
+        <v>0.8502718971426</v>
       </c>
       <c r="E26" t="n">
-        <v>39.8440576150202</v>
+        <v>5.4607065530997</v>
       </c>
       <c r="F26" t="n">
-        <v>4.584167616318433</v>
+        <v>0.4426932116861</v>
       </c>
       <c r="G26" t="n">
-        <v>4.552461656570133</v>
+        <v>0.3189536370345</v>
       </c>
       <c r="H26" t="n">
-        <v>0.3363481283948622</v>
+        <v>0.8814050971143725</v>
       </c>
       <c r="I26" t="n">
-        <v>0.5742849347690112</v>
+        <v>0.742088621041176</v>
       </c>
       <c r="J26" t="n">
-        <v>0.04119993430811005</v>
+        <v>0.005903910494283782</v>
       </c>
       <c r="K26" t="n">
-        <v>0.2332035690559487</v>
+        <v>0.0292460485959992</v>
       </c>
       <c r="L26" t="n">
-        <v>0.04140880397240844</v>
+        <v>0.0006558076291523554</v>
       </c>
       <c r="M26" t="n">
-        <v>0.04162423765643203</v>
+        <v>0.0008996216794094675</v>
       </c>
       <c r="N26" t="n">
-        <v>0.002137836280055393</v>
+        <v>0.0003954003214294751</v>
       </c>
       <c r="O26" t="n">
-        <v>0.004594199489270355</v>
+        <v>0.004041616023135867</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -1995,7 +1995,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2007,40 +2007,40 @@
         <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>4.449146714767501</v>
+        <v>0.8315244011495001</v>
       </c>
       <c r="E27" t="n">
-        <v>38.67817877769927</v>
+        <v>5.49517057619</v>
       </c>
       <c r="F27" t="n">
-        <v>4.347928409348667</v>
+        <v>0.4480075349028334</v>
       </c>
       <c r="G27" t="n">
-        <v>4.311858192818266</v>
+        <v>0.3096465552448</v>
       </c>
       <c r="H27" t="n">
-        <v>0.3442241053826145</v>
+        <v>0.8797687639479914</v>
       </c>
       <c r="I27" t="n">
-        <v>0.5789730031495357</v>
+        <v>0.7223099849766842</v>
       </c>
       <c r="J27" t="n">
-        <v>0.03135161191576255</v>
+        <v>0.008924532141761143</v>
       </c>
       <c r="K27" t="n">
-        <v>0.1721826596775453</v>
+        <v>0.01489261192088886</v>
       </c>
       <c r="L27" t="n">
-        <v>0.03118676514337875</v>
+        <v>0.00251770273208399</v>
       </c>
       <c r="M27" t="n">
-        <v>0.03277733145456132</v>
+        <v>0.001786406062948128</v>
       </c>
       <c r="N27" t="n">
-        <v>0.001632848956886914</v>
+        <v>0.0007436882674003955</v>
       </c>
       <c r="O27" t="n">
-        <v>0.00456913524231088</v>
+        <v>0.005611451055575447</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2054,7 +2054,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2066,43 +2066,43 @@
         <v>3</v>
       </c>
       <c r="D28" t="n">
-        <v>4.480196253950034</v>
+        <v>0.7225773738886001</v>
       </c>
       <c r="E28" t="n">
-        <v>38.89223448794053</v>
+        <v>5.452208487349799</v>
       </c>
       <c r="F28" t="n">
-        <v>4.378142004008133</v>
+        <v>0.4472464966468</v>
       </c>
       <c r="G28" t="n">
-        <v>4.344089959168966</v>
+        <v>0.3135579154232334</v>
       </c>
       <c r="H28" t="n">
-        <v>0.3427342928399741</v>
+        <v>0.8613959983095422</v>
       </c>
       <c r="I28" t="n">
-        <v>0.5839717434300823</v>
+        <v>0.8094781804549888</v>
       </c>
       <c r="J28" t="n">
-        <v>0.03348693805469789</v>
+        <v>0.006392578699177021</v>
       </c>
       <c r="K28" t="n">
-        <v>0.2008306145023352</v>
+        <v>0.03434962783607208</v>
       </c>
       <c r="L28" t="n">
-        <v>0.03296962066273203</v>
+        <v>0.0007994427614239256</v>
       </c>
       <c r="M28" t="n">
-        <v>0.03573225124601732</v>
+        <v>0.0008496145493271741</v>
       </c>
       <c r="N28" t="n">
-        <v>0.002119665720671422</v>
+        <v>0.001506649409099997</v>
       </c>
       <c r="O28" t="n">
-        <v>0.007700102234067678</v>
+        <v>0.002192561491826783</v>
       </c>
       <c r="P28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -2113,57 +2113,883 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>geant</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>3</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.7509228569232</v>
+      </c>
+      <c r="E29" t="n">
+        <v>5.476798487561567</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.4530580908306333</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.3096083548637666</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.8667797937050526</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.7498925451143607</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.006005240601259012</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0.02169411228162643</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0.002751827371387717</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0.0001239548096339272</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0.001177476155245675</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0.005477748418061815</v>
+      </c>
+      <c r="P29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>ST-Adaptive-Ensemble-RL</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>sdn</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>persistence</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>3</v>
+      </c>
+      <c r="D30" t="n">
+        <v>26.55449157545777</v>
+      </c>
+      <c r="E30" t="n">
+        <v>90.96799341654842</v>
+      </c>
+      <c r="F30" t="n">
+        <v>26.42186862643311</v>
+      </c>
+      <c r="G30" t="n">
+        <v>25.69528161983637</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.2110912108471329</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0.4498484483944032</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Persistence</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>branch_xgboost</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" t="n">
+        <v>5.501746132110231</v>
+      </c>
+      <c r="E31" t="n">
+        <v>43.50135691079012</v>
+      </c>
+      <c r="F31" t="n">
+        <v>5.400941108775661</v>
+      </c>
+      <c r="G31" t="n">
+        <v>5.38897000852714</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.3104524120407648</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.5979225042188075</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0.03648634416566095</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0.1800025294142001</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0.03583735584964644</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0.03555507731483454</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0.002514829252129105</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0.008006618946304844</v>
+      </c>
+      <c r="P31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>branch_lightgbm_res</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" t="n">
+        <v>4.725293687942619</v>
+      </c>
+      <c r="E32" t="n">
+        <v>40.09050711039001</v>
+      </c>
+      <c r="F32" t="n">
+        <v>4.622366665383944</v>
+      </c>
+      <c r="G32" t="n">
+        <v>4.58088827254178</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.3346154045021904</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.5685760891694658</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0.04001095344222513</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0.2356779729660841</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0.04040968708202303</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0.04102459753013328</v>
+      </c>
+      <c r="N32" t="n">
+        <v>0.002412511766822248</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0.003194804001046742</v>
+      </c>
+      <c r="P32" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>LightGBM-Residual</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>branch_stwaveformer</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" t="n">
+        <v>15.05727505024088</v>
+      </c>
+      <c r="E33" t="n">
+        <v>64.31187253033912</v>
+      </c>
+      <c r="F33" t="n">
+        <v>14.95331586609725</v>
+      </c>
+      <c r="G33" t="n">
+        <v>14.62828864718621</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0.3033576975106618</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.7939136373143997</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0.3879300898569781</v>
+      </c>
+      <c r="K33" t="n">
+        <v>1.442674289781311</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0.3902316522193149</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0.3791228986791557</v>
+      </c>
+      <c r="N33" t="n">
+        <v>0.007868257797702578</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0.006935287930042821</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>ST-WaveFormer</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>branch_odgraphformer</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" t="n">
+        <v>10.82378673206354</v>
+      </c>
+      <c r="E34" t="n">
+        <v>60.98440293556504</v>
+      </c>
+      <c r="F34" t="n">
+        <v>10.71875904785843</v>
+      </c>
+      <c r="G34" t="n">
+        <v>10.55165324861514</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.2656305682531275</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0.653468604478941</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0.5172167404793825</v>
+      </c>
+      <c r="K34" t="n">
+        <v>1.426460798016727</v>
+      </c>
+      <c r="L34" t="n">
+        <v>0.5149674442874014</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0.4916759040166223</v>
+      </c>
+      <c r="N34" t="n">
+        <v>0.00122086714363905</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0.01292813018908067</v>
+      </c>
+      <c r="P34" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>OD-GraphFormer</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>v3_static</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" t="n">
+        <v>4.016685571412967</v>
+      </c>
+      <c r="E35" t="n">
+        <v>38.12959362032276</v>
+      </c>
+      <c r="F35" t="n">
+        <v>3.9141140577925</v>
+      </c>
+      <c r="G35" t="n">
+        <v>3.881554694383667</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.3216286447809846</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.6358823934634544</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0.0511924947251717</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0.2919558767863844</v>
+      </c>
+      <c r="L35" t="n">
+        <v>0.05138622364983586</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0.05120899677502607</v>
+      </c>
+      <c r="N35" t="n">
+        <v>0.002258133129645119</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0.002740557556229231</v>
+      </c>
+      <c r="P35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>ST-Adaptive-Ensemble v3 (static)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>static_k4</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>3</v>
+      </c>
+      <c r="D36" t="n">
+        <v>4.0006725430085</v>
+      </c>
+      <c r="E36" t="n">
+        <v>38.04336307929087</v>
+      </c>
+      <c r="F36" t="n">
+        <v>3.898104438271266</v>
+      </c>
+      <c r="G36" t="n">
+        <v>3.865385824036534</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0.3221728402357322</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.6361394316594257</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.05083442098161815</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0.2936563955059048</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0.05101751928635763</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0.05081318515054815</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0.002170762595070282</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0.002791217678190753</v>
+      </c>
+      <c r="P36" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Static K=4</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>static_k3</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" t="n">
+        <v>4.684722348874001</v>
+      </c>
+      <c r="E37" t="n">
+        <v>39.83803320540737</v>
+      </c>
+      <c r="F37" t="n">
+        <v>4.582328381558233</v>
+      </c>
+      <c r="G37" t="n">
+        <v>4.553032977087266</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0.3361538283555277</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.5760268776804347</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0.04131775529316326</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0.2329841362440988</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0.04150812133718134</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0.04148202553812069</v>
+      </c>
+      <c r="N37" t="n">
+        <v>0.002092411740696855</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0.004240845807268545</v>
+      </c>
+      <c r="P37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Static K=3 (nhánh RL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>hedge</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" t="n">
+        <v>4.542170142965533</v>
+      </c>
+      <c r="E38" t="n">
+        <v>39.2482763158854</v>
+      </c>
+      <c r="F38" t="n">
+        <v>4.439539794282</v>
+      </c>
+      <c r="G38" t="n">
+        <v>4.422377569527034</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.3365139811403686</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.5854458781691547</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0.03842453494253652</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0.2001784443270455</v>
+      </c>
+      <c r="L38" t="n">
+        <v>0.03870985882774151</v>
+      </c>
+      <c r="M38" t="n">
+        <v>0.03720438800025542</v>
+      </c>
+      <c r="N38" t="n">
+        <v>0.001478039886136305</v>
+      </c>
+      <c r="O38" t="n">
+        <v>0.003967245799738929</v>
+      </c>
+      <c r="P38" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Hedge</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>hedge_floor</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" t="n">
+        <v>4.542170142965533</v>
+      </c>
+      <c r="E39" t="n">
+        <v>39.2482763158854</v>
+      </c>
+      <c r="F39" t="n">
+        <v>4.439539794282</v>
+      </c>
+      <c r="G39" t="n">
+        <v>4.422377569527034</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.3365139811403686</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.5854458781691547</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0.03842453494253652</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0.2001784443270455</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0.03870985882774151</v>
+      </c>
+      <c r="M39" t="n">
+        <v>0.03720438800025542</v>
+      </c>
+      <c r="N39" t="n">
+        <v>0.001478039886136305</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0.003967245799738929</v>
+      </c>
+      <c r="P39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Hedge + sàn</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>context_gate</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>3</v>
+      </c>
+      <c r="D40" t="n">
+        <v>4.686588991352133</v>
+      </c>
+      <c r="E40" t="n">
+        <v>39.8440576150202</v>
+      </c>
+      <c r="F40" t="n">
+        <v>4.584167616318433</v>
+      </c>
+      <c r="G40" t="n">
+        <v>4.552461656570133</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0.3363481283948622</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.5742849347690112</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0.04119993430811005</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0.2332035690559487</v>
+      </c>
+      <c r="L40" t="n">
+        <v>0.04140880397240844</v>
+      </c>
+      <c r="M40" t="n">
+        <v>0.04162423765643203</v>
+      </c>
+      <c r="N40" t="n">
+        <v>0.002137836280055393</v>
+      </c>
+      <c r="O40" t="n">
+        <v>0.004594199489270355</v>
+      </c>
+      <c r="P40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Cổng MLP ngữ cảnh v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>rl_sup</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" t="n">
+        <v>4.449146714767501</v>
+      </c>
+      <c r="E41" t="n">
+        <v>38.67817877769927</v>
+      </c>
+      <c r="F41" t="n">
+        <v>4.347928409348667</v>
+      </c>
+      <c r="G41" t="n">
+        <v>4.311858192818266</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.3442241053826145</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0.5789730031495357</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0.03135161191576255</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0.1721826596775453</v>
+      </c>
+      <c r="L41" t="n">
+        <v>0.03118676514337875</v>
+      </c>
+      <c r="M41" t="n">
+        <v>0.03277733145456132</v>
+      </c>
+      <c r="N41" t="n">
+        <v>0.001632848956886914</v>
+      </c>
+      <c r="O41" t="n">
+        <v>0.00456913524231088</v>
+      </c>
+      <c r="P41" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Gate giám sát (γ=0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>rl_sac</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>3</v>
+      </c>
+      <c r="D42" t="n">
+        <v>4.480196253950034</v>
+      </c>
+      <c r="E42" t="n">
+        <v>38.89223448794053</v>
+      </c>
+      <c r="F42" t="n">
+        <v>4.378142004008133</v>
+      </c>
+      <c r="G42" t="n">
+        <v>4.344089959168966</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0.3427342928399741</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0.5839717434300823</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0.03348693805469789</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0.2008306145023352</v>
+      </c>
+      <c r="L42" t="n">
+        <v>0.03296962066273203</v>
+      </c>
+      <c r="M42" t="n">
+        <v>0.03573225124601732</v>
+      </c>
+      <c r="N42" t="n">
+        <v>0.002119665720671422</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0.007700102234067678</v>
+      </c>
+      <c r="P42" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>RL-Gate (SAC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
         <is>
           <t>final</t>
         </is>
       </c>
-      <c r="C29" t="n">
-        <v>3</v>
-      </c>
-      <c r="D29" t="n">
+      <c r="C43" t="n">
+        <v>3</v>
+      </c>
+      <c r="D43" t="n">
         <v>4.480196253950034</v>
       </c>
-      <c r="E29" t="n">
+      <c r="E43" t="n">
         <v>38.89223448794053</v>
       </c>
-      <c r="F29" t="n">
+      <c r="F43" t="n">
         <v>4.378142004008133</v>
       </c>
-      <c r="G29" t="n">
+      <c r="G43" t="n">
         <v>4.344089959168966</v>
       </c>
-      <c r="H29" t="n">
+      <c r="H43" t="n">
         <v>0.3427342928399741</v>
       </c>
-      <c r="I29" t="n">
+      <c r="I43" t="n">
         <v>0.5839717434300823</v>
       </c>
-      <c r="J29" t="n">
+      <c r="J43" t="n">
         <v>0.03348693805469789</v>
       </c>
-      <c r="K29" t="n">
+      <c r="K43" t="n">
         <v>0.2008306145023352</v>
       </c>
-      <c r="L29" t="n">
+      <c r="L43" t="n">
         <v>0.03296962066273203</v>
       </c>
-      <c r="M29" t="n">
+      <c r="M43" t="n">
         <v>0.03573225124601732</v>
       </c>
-      <c r="N29" t="n">
+      <c r="N43" t="n">
         <v>0.002119665720671422</v>
       </c>
-      <c r="O29" t="n">
+      <c r="O43" t="n">
         <v>0.007700102234067678</v>
       </c>
-      <c r="P29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q29" t="inlineStr">
+      <c r="P43" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q43" t="inlineStr">
         <is>
           <t>ST-Adaptive-Ensemble-RL</t>
         </is>
@@ -2180,7 +3006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2745,7 +3571,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2757,40 +3583,40 @@
         <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>4.8276139688106</v>
+        <v>0.8412722016658769</v>
       </c>
       <c r="E10" t="n">
-        <v>41.5047214284323</v>
+        <v>6.700048338662969</v>
       </c>
       <c r="F10" t="n">
-        <v>4.748738791231708</v>
+        <v>0.5339038520291073</v>
       </c>
       <c r="G10" t="n">
-        <v>4.748759486366427</v>
+        <v>0.4130891701636559</v>
       </c>
       <c r="H10" t="n">
-        <v>0.2963983477427541</v>
+        <v>0.8264881986127447</v>
       </c>
       <c r="I10" t="n">
-        <v>0.5299587290167037</v>
+        <v>0.7695749586861611</v>
       </c>
       <c r="J10" t="n">
-        <v>0.2357659810412736</v>
+        <v>0.04522018766115047</v>
       </c>
       <c r="K10" t="n">
-        <v>1.023521497138683</v>
+        <v>0.4709433489306898</v>
       </c>
       <c r="L10" t="n">
-        <v>0.2375486340469883</v>
+        <v>0.04946887346935822</v>
       </c>
       <c r="M10" t="n">
-        <v>0.2362353370503212</v>
+        <v>0.05081243931622949</v>
       </c>
       <c r="N10" t="n">
-        <v>0.006027497320855425</v>
+        <v>0.01893237121465203</v>
       </c>
       <c r="O10" t="n">
-        <v>0.01153529849583505</v>
+        <v>0.03946966795537322</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -2804,7 +3630,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2816,40 +3642,40 @@
         <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>10.66293271400805</v>
+        <v>0.7778650781914038</v>
       </c>
       <c r="E11" t="n">
-        <v>60.30897322814824</v>
+        <v>5.81166096118405</v>
       </c>
       <c r="F11" t="n">
-        <v>10.5588699804009</v>
+        <v>0.514531533423087</v>
       </c>
       <c r="G11" t="n">
-        <v>10.40103781037437</v>
+        <v>0.3100588220072919</v>
       </c>
       <c r="H11" t="n">
-        <v>0.2632649427674279</v>
+        <v>0.8683078029040253</v>
       </c>
       <c r="I11" t="n">
-        <v>0.6470081480990179</v>
+        <v>0.6321458983153531</v>
       </c>
       <c r="J11" t="n">
-        <v>0.08053701985678052</v>
+        <v>0.002083426505635926</v>
       </c>
       <c r="K11" t="n">
-        <v>0.2267106013798933</v>
+        <v>0.09659267239247618</v>
       </c>
       <c r="L11" t="n">
-        <v>0.08002285928659564</v>
+        <v>0.003925570152492878</v>
       </c>
       <c r="M11" t="n">
-        <v>0.06990591943031775</v>
+        <v>0.001534919944643368</v>
       </c>
       <c r="N11" t="n">
-        <v>0.002663265318122867</v>
+        <v>0.001776398938480791</v>
       </c>
       <c r="O11" t="n">
-        <v>0.001422903613711275</v>
+        <v>0.006154925877781812</v>
       </c>
       <c r="P11" t="n">
         <v>0</v>
@@ -2863,7 +3689,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2875,40 +3701,40 @@
         <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>10.9102780209387</v>
+        <v>0.7770090187044597</v>
       </c>
       <c r="E12" t="n">
-        <v>61.18399339636263</v>
+        <v>6.002283156188509</v>
       </c>
       <c r="F12" t="n">
-        <v>10.80425328520641</v>
+        <v>0.513613217856743</v>
       </c>
       <c r="G12" t="n">
-        <v>10.63499236387419</v>
+        <v>0.3096060580019913</v>
       </c>
       <c r="H12" t="n">
-        <v>0.2635857497749368</v>
+        <v>0.8679675444598273</v>
       </c>
       <c r="I12" t="n">
-        <v>0.6659195441296032</v>
+        <v>0.6313369926464928</v>
       </c>
       <c r="J12" t="n">
-        <v>0.066160960598211</v>
+        <v>0.008698157221611111</v>
       </c>
       <c r="K12" t="n">
-        <v>0.1883156720439629</v>
+        <v>0.1608085243599109</v>
       </c>
       <c r="L12" t="n">
-        <v>0.06655299041987504</v>
+        <v>0.008116798029081896</v>
       </c>
       <c r="M12" t="n">
-        <v>0.04785879943660532</v>
+        <v>0.001082225328525832</v>
       </c>
       <c r="N12" t="n">
-        <v>0.00395845662169573</v>
+        <v>0.001721541742660038</v>
       </c>
       <c r="O12" t="n">
-        <v>0.01444244036559092</v>
+        <v>0.01484493183029602</v>
       </c>
       <c r="P12" t="n">
         <v>0</v>
@@ -2922,7 +3748,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2934,40 +3760,40 @@
         <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>4.6007980620559</v>
+        <v>0.7247457596141333</v>
       </c>
       <c r="E13" t="n">
-        <v>39.4685735956757</v>
+        <v>5.4558972742523</v>
       </c>
       <c r="F13" t="n">
-        <v>4.497778798865401</v>
+        <v>0.4471611844811667</v>
       </c>
       <c r="G13" t="n">
-        <v>4.483965509299467</v>
+        <v>0.3135538313407667</v>
       </c>
       <c r="H13" t="n">
-        <v>0.3366507029696833</v>
+        <v>0.8617371596332469</v>
       </c>
       <c r="I13" t="n">
-        <v>0.582159349679667</v>
+        <v>0.8075838095144151</v>
       </c>
       <c r="J13" t="n">
-        <v>0.03924523452740855</v>
+        <v>0.004811167879593192</v>
       </c>
       <c r="K13" t="n">
-        <v>0.2237184556650453</v>
+        <v>0.04128401614411725</v>
       </c>
       <c r="L13" t="n">
-        <v>0.03949077697060992</v>
+        <v>0.001759877318616768</v>
       </c>
       <c r="M13" t="n">
-        <v>0.03871445401052525</v>
+        <v>0.0005885793199760678</v>
       </c>
       <c r="N13" t="n">
-        <v>0.001850556307376831</v>
+        <v>0.001668643552544099</v>
       </c>
       <c r="O13" t="n">
-        <v>0.003245605516320773</v>
+        <v>0.002044643598944698</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
@@ -2981,7 +3807,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2993,40 +3819,40 @@
         <v>3</v>
       </c>
       <c r="D14" t="n">
-        <v>4.528418422798134</v>
+        <v>0.7228733764374665</v>
       </c>
       <c r="E14" t="n">
-        <v>39.09603904405284</v>
+        <v>5.452157136310833</v>
       </c>
       <c r="F14" t="n">
-        <v>4.4259005183743</v>
+        <v>0.4471955007365666</v>
       </c>
       <c r="G14" t="n">
-        <v>4.389191853846733</v>
+        <v>0.3136546782959</v>
       </c>
       <c r="H14" t="n">
-        <v>0.3421658448997631</v>
+        <v>0.8614258152017199</v>
       </c>
       <c r="I14" t="n">
-        <v>0.5692215955020613</v>
+        <v>0.8097562288404866</v>
       </c>
       <c r="J14" t="n">
-        <v>0.0162723717959731</v>
+        <v>0.006138289059896838</v>
       </c>
       <c r="K14" t="n">
-        <v>0.1207024858161245</v>
+        <v>0.03366806413381793</v>
       </c>
       <c r="L14" t="n">
-        <v>0.01652362515098457</v>
+        <v>0.0007867838598981026</v>
       </c>
       <c r="M14" t="n">
-        <v>0.01763783668073158</v>
+        <v>0.0007313476638653268</v>
       </c>
       <c r="N14" t="n">
-        <v>0.001514510517106802</v>
+        <v>0.001465533828970079</v>
       </c>
       <c r="O14" t="n">
-        <v>0.00548192115092797</v>
+        <v>0.002259692767003958</v>
       </c>
       <c r="P14" t="n">
         <v>0</v>
@@ -3040,7 +3866,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3052,40 +3878,40 @@
         <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>4.710557639548266</v>
+        <v>0.7218451636614334</v>
       </c>
       <c r="E15" t="n">
-        <v>40.06596057594567</v>
+        <v>5.455012669519333</v>
       </c>
       <c r="F15" t="n">
-        <v>4.608354158853033</v>
+        <v>0.4471953363100333</v>
       </c>
       <c r="G15" t="n">
-        <v>4.589994634922399</v>
+        <v>0.3132705326157333</v>
       </c>
       <c r="H15" t="n">
-        <v>0.3321333617750766</v>
+        <v>0.8612424204224908</v>
       </c>
       <c r="I15" t="n">
-        <v>0.5812170010577616</v>
+        <v>0.8094240791732087</v>
       </c>
       <c r="J15" t="n">
-        <v>0.1769022240669252</v>
+        <v>0.005877267269421888</v>
       </c>
       <c r="K15" t="n">
-        <v>0.787068196298402</v>
+        <v>0.03145793899763993</v>
       </c>
       <c r="L15" t="n">
-        <v>0.1763398443973145</v>
+        <v>0.000585589696054073</v>
       </c>
       <c r="M15" t="n">
-        <v>0.177536843462079</v>
+        <v>0.000801606758211442</v>
       </c>
       <c r="N15" t="n">
-        <v>0.004822580596551231</v>
+        <v>0.001420777978255195</v>
       </c>
       <c r="O15" t="n">
-        <v>0.008334709652361447</v>
+        <v>0.001784030015620982</v>
       </c>
       <c r="P15" t="n">
         <v>0</v>
@@ -3099,7 +3925,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3111,40 +3937,40 @@
         <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>10.82378673206354</v>
+        <v>0.7856831775612649</v>
       </c>
       <c r="E16" t="n">
-        <v>60.98440293556504</v>
+        <v>5.887070317139143</v>
       </c>
       <c r="F16" t="n">
-        <v>10.71875904785843</v>
+        <v>0.5178367351444001</v>
       </c>
       <c r="G16" t="n">
-        <v>10.55165324861514</v>
+        <v>0.3107024173756095</v>
       </c>
       <c r="H16" t="n">
-        <v>0.2656305682531275</v>
+        <v>0.8694401492276453</v>
       </c>
       <c r="I16" t="n">
-        <v>0.653468604478941</v>
+        <v>0.6240313550206674</v>
       </c>
       <c r="J16" t="n">
-        <v>0.5172167404793825</v>
+        <v>0.01041224897936075</v>
       </c>
       <c r="K16" t="n">
-        <v>1.426460798016727</v>
+        <v>0.2274492561295375</v>
       </c>
       <c r="L16" t="n">
-        <v>0.5149674442874014</v>
+        <v>0.007818188448588366</v>
       </c>
       <c r="M16" t="n">
-        <v>0.4916759040166223</v>
+        <v>0.0003525583492634219</v>
       </c>
       <c r="N16" t="n">
-        <v>0.00122086714363905</v>
+        <v>0.002671004988153148</v>
       </c>
       <c r="O16" t="n">
-        <v>0.01292813018908067</v>
+        <v>0.01458200086210178</v>
       </c>
       <c r="P16" t="n">
         <v>0</v>
@@ -3158,57 +3984,529 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>geant</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>rl_sac</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.7225773738886001</v>
+      </c>
+      <c r="E17" t="n">
+        <v>5.452208487349799</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.4472464966468</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.3135579154232334</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.8613959983095422</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.8094781804549888</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.006392578699177021</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.03434962783607208</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.0007994427614239256</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.0008496145493271741</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0.001506649409099997</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.002192561491826783</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>RL-Gate đầy đủ</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>sdn</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>odgraphformer_no_residual</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" t="n">
+        <v>4.8276139688106</v>
+      </c>
+      <c r="E18" t="n">
+        <v>41.5047214284323</v>
+      </c>
+      <c r="F18" t="n">
+        <v>4.748738791231708</v>
+      </c>
+      <c r="G18" t="n">
+        <v>4.748759486366427</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.2963983477427541</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.5299587290167037</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.2357659810412736</v>
+      </c>
+      <c r="K18" t="n">
+        <v>1.023521497138683</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0.2375486340469883</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.2362353370503212</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0.006027497320855425</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0.01153529849583505</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>OD-GraphFormer: bỏ mục tiêu phần dư</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>odgraphformer_no_route</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>3</v>
+      </c>
+      <c r="D19" t="n">
+        <v>10.66293271400805</v>
+      </c>
+      <c r="E19" t="n">
+        <v>60.30897322814824</v>
+      </c>
+      <c r="F19" t="n">
+        <v>10.5588699804009</v>
+      </c>
+      <c r="G19" t="n">
+        <v>10.40103781037437</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.2632649427674279</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.6470081480990179</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.08053701985678052</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.2267106013798933</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0.08002285928659564</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0.06990591943031775</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0.002663265318122867</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.001422903613711275</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>OD-GraphFormer: bỏ A_route</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>odgraphformer_no_spatial_attn</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" t="n">
+        <v>10.9102780209387</v>
+      </c>
+      <c r="E20" t="n">
+        <v>61.18399339636263</v>
+      </c>
+      <c r="F20" t="n">
+        <v>10.80425328520641</v>
+      </c>
+      <c r="G20" t="n">
+        <v>10.63499236387419</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.2635857497749368</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.6659195441296032</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.066160960598211</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.1883156720439629</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0.06655299041987504</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0.04785879943660532</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0.00395845662169573</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0.01444244036559092</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>OD-GraphFormer: bỏ attention giữa luồng</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>rl_sac_no_gnn</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" t="n">
+        <v>4.6007980620559</v>
+      </c>
+      <c r="E21" t="n">
+        <v>39.4685735956757</v>
+      </c>
+      <c r="F21" t="n">
+        <v>4.497778798865401</v>
+      </c>
+      <c r="G21" t="n">
+        <v>4.483965509299467</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.3366507029696833</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.582159349679667</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.03924523452740855</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.2237184556650453</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0.03949077697060992</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0.03871445401052525</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0.001850556307376831</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0.003245605516320773</v>
+      </c>
+      <c r="P21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>RL-Gate: bỏ GNN</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>rl_sac_no_floor</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" t="n">
+        <v>4.528418422798134</v>
+      </c>
+      <c r="E22" t="n">
+        <v>39.09603904405284</v>
+      </c>
+      <c r="F22" t="n">
+        <v>4.4259005183743</v>
+      </c>
+      <c r="G22" t="n">
+        <v>4.389191853846733</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.3421658448997631</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.5692215955020613</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.0162723717959731</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0.1207024858161245</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0.01652362515098457</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0.01763783668073158</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0.001514510517106802</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0.00548192115092797</v>
+      </c>
+      <c r="P22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>RL-Gate: bỏ ràng buộc sàn</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>rl_sac_no_oof</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" t="n">
+        <v>4.710557639548266</v>
+      </c>
+      <c r="E23" t="n">
+        <v>40.06596057594567</v>
+      </c>
+      <c r="F23" t="n">
+        <v>4.608354158853033</v>
+      </c>
+      <c r="G23" t="n">
+        <v>4.589994634922399</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.3321333617750766</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.5812170010577616</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.1769022240669252</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0.787068196298402</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0.1763398443973145</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0.177536843462079</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0.004822580596551231</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0.008334709652361447</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>RL-Gate: không dùng OOF</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>branch_odgraphformer</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" t="n">
+        <v>10.82378673206354</v>
+      </c>
+      <c r="E24" t="n">
+        <v>60.98440293556504</v>
+      </c>
+      <c r="F24" t="n">
+        <v>10.71875904785843</v>
+      </c>
+      <c r="G24" t="n">
+        <v>10.55165324861514</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.2656305682531275</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.653468604478941</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.5172167404793825</v>
+      </c>
+      <c r="K24" t="n">
+        <v>1.426460798016727</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0.5149674442874014</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0.4916759040166223</v>
+      </c>
+      <c r="N24" t="n">
+        <v>0.00122086714363905</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0.01292813018908067</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>OD-GraphFormer đầy đủ</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
         <is>
           <t>rl_sac</t>
         </is>
       </c>
-      <c r="C17" t="n">
-        <v>3</v>
-      </c>
-      <c r="D17" t="n">
+      <c r="C25" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" t="n">
         <v>4.480196253950034</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E25" t="n">
         <v>38.89223448794053</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F25" t="n">
         <v>4.378142004008133</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G25" t="n">
         <v>4.344089959168966</v>
       </c>
-      <c r="H17" t="n">
+      <c r="H25" t="n">
         <v>0.3427342928399741</v>
       </c>
-      <c r="I17" t="n">
+      <c r="I25" t="n">
         <v>0.5839717434300823</v>
       </c>
-      <c r="J17" t="n">
+      <c r="J25" t="n">
         <v>0.03348693805469789</v>
       </c>
-      <c r="K17" t="n">
+      <c r="K25" t="n">
         <v>0.2008306145023352</v>
       </c>
-      <c r="L17" t="n">
+      <c r="L25" t="n">
         <v>0.03296962066273203</v>
       </c>
-      <c r="M17" t="n">
+      <c r="M25" t="n">
         <v>0.03573225124601732</v>
       </c>
-      <c r="N17" t="n">
+      <c r="N25" t="n">
         <v>0.002119665720671422</v>
       </c>
-      <c r="O17" t="n">
+      <c r="O25" t="n">
         <v>0.007700102234067678</v>
       </c>
-      <c r="P17" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" t="inlineStr">
+      <c r="P25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="inlineStr">
         <is>
           <t>RL-Gate đầy đủ</t>
         </is>
@@ -3225,7 +4523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3298,7 +4596,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3315,37 +4613,37 @@
         <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>4.480196253950034</v>
+        <v>0.7509228569232</v>
       </c>
       <c r="F2" t="n">
-        <v>4.016685571412967</v>
+        <v>0.7235077901182333</v>
       </c>
       <c r="G2" t="n">
-        <v>11.53963073026936</v>
+        <v>3.789187508331682</v>
       </c>
       <c r="H2" t="n">
-        <v>38.40527799254714</v>
+        <v>43.2856381286385</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0006772933045598784</v>
+        <v>0.0005332917124479696</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>40.08633356203017</v>
+        <v>1.037834748528587</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3362,28 +4660,24 @@
         <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>4.480196253950034</v>
+        <v>0.7509228569232</v>
       </c>
       <c r="F3" t="n">
-        <v>4.542170142965533</v>
+        <v>0.7509228569232</v>
       </c>
       <c r="G3" t="n">
-        <v>-1.364411439132884</v>
-      </c>
-      <c r="H3" t="n">
-        <v>-8.498071192783728</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.01356598098243242</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>-2.676809159576517</v>
+        <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
@@ -3392,7 +4686,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3409,37 +4703,37 @@
         <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>4.480196253950034</v>
+        <v>0.7225773738886001</v>
       </c>
       <c r="F4" t="n">
-        <v>4.016685571412967</v>
+        <v>0.7235077901182333</v>
       </c>
       <c r="G4" t="n">
-        <v>11.53963073026936</v>
+        <v>-0.1285979560055828</v>
       </c>
       <c r="H4" t="n">
-        <v>38.40527799254714</v>
+        <v>-0.8860603210555734</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0006772933045598784</v>
+        <v>0.469063397337544</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K4" t="n">
-        <v>40.08633356203017</v>
+        <v>-0.3156124308625227</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3456,28 +4750,28 @@
         <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>4.480196253950034</v>
+        <v>0.7225773738886001</v>
       </c>
       <c r="F5" t="n">
-        <v>4.542170142965533</v>
+        <v>0.7509228569232</v>
       </c>
       <c r="G5" t="n">
-        <v>-1.364411439132884</v>
+        <v>-3.77475299536647</v>
       </c>
       <c r="H5" t="n">
-        <v>-8.498071192783728</v>
+        <v>-64.98215176605167</v>
       </c>
       <c r="I5" t="n">
-        <v>0.01356598098243242</v>
+        <v>0.0002367323368356586</v>
       </c>
       <c r="J5" t="n">
         <v>3</v>
       </c>
       <c r="K5" t="n">
-        <v>-2.676809159576517</v>
+        <v>-1.048095862852264</v>
       </c>
       <c r="L5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
         <v>0</v>
@@ -3486,7 +4780,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>sdn</t>
+          <t>geant</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3503,37 +4797,37 @@
         <v>3</v>
       </c>
       <c r="E6" t="n">
-        <v>4.480196253950034</v>
+        <v>0.7225773738886001</v>
       </c>
       <c r="F6" t="n">
-        <v>4.449146714767501</v>
+        <v>0.8315244011495001</v>
       </c>
       <c r="G6" t="n">
-        <v>0.6978762709594077</v>
+        <v>-13.10208420947017</v>
       </c>
       <c r="H6" t="n">
-        <v>3.1094933503205</v>
+        <v>-34.89577546386102</v>
       </c>
       <c r="I6" t="n">
-        <v>0.08972259348788525</v>
+        <v>0.0008201999230144778</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K6" t="n">
-        <v>5.456195002320371</v>
+        <v>-1.134991647514192</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>abilene</t>
+          <t>sdn</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3550,37 +4844,37 @@
         <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>1.846252116050033</v>
+        <v>4.480196253950034</v>
       </c>
       <c r="F7" t="n">
-        <v>1.847143500100633</v>
+        <v>4.016685571412967</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.0482574337376418</v>
+        <v>11.53963073026936</v>
       </c>
       <c r="H7" t="n">
-        <v>-7.134252375054712</v>
+        <v>38.40527799254714</v>
       </c>
       <c r="I7" t="n">
-        <v>0.01908661415596488</v>
+        <v>0.0006772933045598784</v>
       </c>
       <c r="J7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>-6.759745617398047</v>
+        <v>40.08633356203017</v>
       </c>
       <c r="L7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>abilene</t>
+          <t>sdn</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3597,37 +4891,37 @@
         <v>3</v>
       </c>
       <c r="E8" t="n">
-        <v>1.846252116050033</v>
+        <v>4.480196253950034</v>
       </c>
       <c r="F8" t="n">
-        <v>1.671145775968867</v>
+        <v>4.542170142965533</v>
       </c>
       <c r="G8" t="n">
-        <v>10.4782205477943</v>
+        <v>-1.364411439132884</v>
       </c>
       <c r="H8" t="n">
-        <v>7.075378820440743</v>
+        <v>-8.498071192783728</v>
       </c>
       <c r="I8" t="n">
-        <v>0.01939635107665707</v>
+        <v>0.01356598098243242</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K8" t="n">
-        <v>8.871957314239927</v>
+        <v>-2.676809159576517</v>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M8" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>abilene</t>
+          <t>sdn</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3644,25 +4938,25 @@
         <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>1.855865671600433</v>
+        <v>4.480196253950034</v>
       </c>
       <c r="F9" t="n">
-        <v>1.847143500100633</v>
+        <v>4.016685571412967</v>
       </c>
       <c r="G9" t="n">
-        <v>0.4721978286648998</v>
+        <v>11.53963073026936</v>
       </c>
       <c r="H9" t="n">
-        <v>2.255318542437188</v>
+        <v>38.40527799254714</v>
       </c>
       <c r="I9" t="n">
-        <v>0.1527859145661754</v>
+        <v>0.0006772933045598784</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>4.852475669319289</v>
+        <v>40.08633356203017</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
@@ -3674,7 +4968,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>abilene</t>
+          <t>sdn</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -3691,77 +4985,312 @@
         <v>3</v>
       </c>
       <c r="E10" t="n">
-        <v>1.855865671600433</v>
+        <v>4.480196253950034</v>
       </c>
       <c r="F10" t="n">
-        <v>1.671145775968867</v>
+        <v>4.542170142965533</v>
       </c>
       <c r="G10" t="n">
-        <v>11.05348786969065</v>
+        <v>-1.364411439132884</v>
       </c>
       <c r="H10" t="n">
-        <v>8.259380745990644</v>
+        <v>-8.498071192783728</v>
       </c>
       <c r="I10" t="n">
-        <v>0.01434437081376579</v>
+        <v>0.01356598098243242</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K10" t="n">
-        <v>9.291061855472298</v>
+        <v>-2.676809159576517</v>
       </c>
       <c r="L10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>sdn</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>rl_sac</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>rl_sup</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4.480196253950034</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4.449146714767501</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.6978762709594077</v>
+      </c>
+      <c r="H11" t="n">
+        <v>3.1094933503205</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.08972259348788525</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>5.456195002320371</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>abilene</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>v3_static</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1.846252116050033</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1.847143500100633</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-0.0482574337376418</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-7.134252375054712</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.01908661415596488</v>
+      </c>
+      <c r="J12" t="n">
+        <v>3</v>
+      </c>
+      <c r="K12" t="n">
+        <v>-6.759745617398047</v>
+      </c>
+      <c r="L12" t="n">
+        <v>3</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>abilene</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>hedge</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1.846252116050033</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1.671145775968867</v>
+      </c>
+      <c r="G13" t="n">
+        <v>10.4782205477943</v>
+      </c>
+      <c r="H13" t="n">
+        <v>7.075378820440743</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.01939635107665707</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>8.871957314239927</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>abilene</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>rl_sac</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>v3_static</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1.855865671600433</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1.847143500100633</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.4721978286648998</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2.255318542437188</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.1527859145661754</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>4.852475669319289</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>abilene</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>rl_sac</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>hedge</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1.855865671600433</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1.671145775968867</v>
+      </c>
+      <c r="G15" t="n">
+        <v>11.05348786969065</v>
+      </c>
+      <c r="H15" t="n">
+        <v>8.259380745990644</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.01434437081376579</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>9.291061855472298</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>abilene</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>rl_sac</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t>rl_sup</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>3</v>
-      </c>
-      <c r="E11" t="n">
+      <c r="D16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" t="n">
         <v>1.855865671600433</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F16" t="n">
         <v>1.810521814871367</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G16" t="n">
         <v>2.504463429085391</v>
       </c>
-      <c r="H11" t="n">
+      <c r="H16" t="n">
         <v>24.58506358836929</v>
       </c>
-      <c r="I11" t="n">
+      <c r="I16" t="n">
         <v>0.001650369437058052</v>
       </c>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="n">
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
         <v>5.442317336115207</v>
       </c>
-      <c r="L11" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" t="n">
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>